<commit_message>
feat: Add data processing and analysis scripts for aluminum output study
- Created Y_Output_cleaned.csv with cleaned output data for provinces from 2015 to 2025.
- Developed step1_data-merge.py to merge output, control, and core explanatory variables into a complete panel dataset.
- Implemented step2.py for descriptive statistics, correlation heatmap, and output trend analysis between treatment and control groups.
- Added step3.py to perform fixed effects regression analysis using PanelOLS and save results.
- Introduced step4.py for DID analysis, including visualization of treatment effects and saving results.
- Developed step5.py to fit a GAM model for nonlinear effects analysis and save results and visualizations.
- Created step6.py for robustness checks, including lagged variable analysis and subsample regression, with results saved for review.
- Added various output files including statistical summaries, plots, and analysis results in both text and image formats.
</commit_message>
<xml_diff>
--- a/Data/Y_Output.xlsx
+++ b/Data/Y_Output.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\statistical-model\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\统计建模\数据\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B646C3-9B2B-4394-B3FA-2BAE01708307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F1B4AA4-E447-49E3-9EB5-67D5C1D2A2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="52">
   <si>
     <t>province_code</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -222,6 +222,14 @@
   </si>
   <si>
     <t>聚汇数据</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>广西统计局</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>云南统计局</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -582,11 +590,11 @@
       <c r="C2">
         <v>2015</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
+      <c r="D2">
+        <v>120.03</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -735,11 +743,11 @@
       <c r="C11">
         <v>2024</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
+      <c r="D11">
+        <v>556.78</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -752,11 +760,11 @@
       <c r="C12">
         <v>2025</v>
       </c>
-      <c r="D12" t="s">
-        <v>11</v>
+      <c r="D12">
+        <v>616.67999999999995</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -922,11 +930,11 @@
       <c r="C22">
         <v>2024</v>
       </c>
-      <c r="D22" t="s">
-        <v>11</v>
+      <c r="D22">
+        <v>293.23</v>
       </c>
       <c r="E22" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>